<commit_message>
Nuevo tipo de evento: FORO
Participación con fecha límite: se guarda como entrega (hora límite,
sin hora = 11:59 PM, estados de vencimiento) pero se muestra con color
violeta, ícono y filtro propios, y botón «Ir al foro» cuando tiene enlace.
Disponible en el editor, la plantilla de Excel y la validación (los
duplicados distinguen foro de trabajo).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQGbJzWknhnvewuJZUfHUT
</commit_message>
<xml_diff>
--- a/public/plantilla-calendario.xlsx
+++ b/public/plantilla-calendario.xlsx
@@ -64,7 +64,7 @@
       <color rgb="00211F18"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +84,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FBEBDC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEE4FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -167,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -198,9 +203,12 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7626,8 +7634,8 @@
   </sheetData>
   <autoFilter ref="A1:H1001"/>
   <dataValidations count="7">
-    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige CLASE, SESION, TRABAJO o ENTREGA." promptTitle="TIPO" prompt="Elige de la lista: CLASE, SESION, TRABAJO o ENTREGA." type="list">
-      <formula1>"CLASE,SESION,TRABAJO,ENTREGA"</formula1>
+    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige CLASE, SESION, TRABAJO, ENTREGA o FORO." promptTitle="TIPO" prompt="Elige de la lista: CLASE, SESION, TRABAJO, ENTREGA o FORO." type="list">
+      <formula1>"CLASE,SESION,TRABAJO,ENTREGA,FORO"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Escribe la fecha como dd/mm/aaaa, por ejemplo 05/10/2026." promptTitle="FECHA" prompt="Formato dd/mm/aaaa. Ejemplo: 05/10/2026." type="date" operator="between">
       <formula1>DATE(2020,1,1)</formula1>
@@ -7660,7 +7668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F36"/>
+  <dimension ref="B2:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -7804,7 +7812,7 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>CLASE o SESION = sesión (azul). TRABAJO o ENTREGA = entrega (naranja).</t>
+          <t>CLASE o SESION = sesión (azul). TRABAJO o ENTREGA = entrega (naranja). FORO = foro (violeta), con hora límite como una entrega.</t>
         </is>
       </c>
     </row>
@@ -8112,113 +8120,140 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="8" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>(vacío)</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>FORO</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Foro: la complejidad de la vida</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>07/03/2027 · 23:59</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>Participación en el foro de la plataforma</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Errores frecuentes</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="10" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>Problema</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="15" t="n"/>
-      <c r="F30" s="10" t="inlineStr">
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="16" t="n"/>
+      <c r="F31" s="10" t="inlineStr">
         <is>
           <t>Cómo corregirlo</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="16" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>Fecha como 35/15/2026</t>
         </is>
       </c>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="14" t="n"/>
-      <c r="E31" s="15" t="n"/>
-      <c r="F31" s="16" t="inlineStr">
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="17" t="inlineStr">
         <is>
           <t>Revisa día y mes. Debe ser una fecha real en formato dd/mm/aaaa.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="16" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>ID_EVENTO repetido</t>
         </is>
       </c>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="14" t="n"/>
-      <c r="E32" s="15" t="n"/>
-      <c r="F32" s="16" t="inlineStr">
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="17" t="inlineStr">
         <is>
           <t>Cada ID aparece una sola vez. En filas nuevas deja la celda vacía.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="16" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>Tipo «REUNION»</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="14" t="n"/>
-      <c r="E33" s="15" t="n"/>
-      <c r="F33" s="16" t="inlineStr">
-        <is>
-          <t>Usa solo CLASE, SESION, TRABAJO o ENTREGA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="16" t="inlineStr">
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="16" t="n"/>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>Usa solo CLASE, SESION, TRABAJO, ENTREGA o FORO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="17" t="inlineStr">
         <is>
           <t>Clase sin hora de inicio</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n"/>
-      <c r="D34" s="14" t="n"/>
-      <c r="E34" s="15" t="n"/>
-      <c r="F34" s="16" t="inlineStr">
+      <c r="C35" s="15" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="E35" s="16" t="n"/>
+      <c r="F35" s="17" t="inlineStr">
         <is>
           <t>Las clases y sesiones necesitan HORA_INICIO.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="16" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="17" t="inlineStr">
         <is>
           <t>Hora fin antes del inicio</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n"/>
-      <c r="D35" s="14" t="n"/>
-      <c r="E35" s="15" t="n"/>
-      <c r="F35" s="16" t="inlineStr">
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="16" t="n"/>
+      <c r="F36" s="17" t="inlineStr">
         <is>
           <t>Corrige HORA_FIN o déjala vacía.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="16" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="17" t="inlineStr">
         <is>
           <t>Link sin https://</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n"/>
-      <c r="D36" s="14" t="n"/>
-      <c r="E36" s="15" t="n"/>
-      <c r="F36" s="16" t="inlineStr">
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="16" t="n"/>
+      <c r="F37" s="17" t="inlineStr">
         <is>
           <t>Copia el enlace completo, empezando por https://</t>
         </is>
@@ -8230,9 +8265,9 @@
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B37:E37"/>
     <mergeCell ref="B34:E34"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B30:E30"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B9:F9"/>

</xml_diff>

<commit_message>
El tipo ENTREGA pasa a ser CUESTIONARIO (verde, ícono de examen)
Cuestionario con fecha límite, color verde, ícono de hoja de examen,
filtro propio y botón «Presentar cuestionario» cuando tiene enlace.
ENTREGA se sigue aceptando como nombre antiguo (Excel y respaldos) y se
guarda como CUESTIONARIO. La migración convierte los eventos existentes
y recalcula su huella para que no aparezcan como modificados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQGbJzWknhnvewuJZUfHUT
</commit_message>
<xml_diff>
--- a/public/plantilla-calendario.xlsx
+++ b/public/plantilla-calendario.xlsx
@@ -7634,8 +7634,8 @@
   </sheetData>
   <autoFilter ref="A1:H1001"/>
   <dataValidations count="7">
-    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige CLASE, SESION, TRABAJO, ENTREGA o FORO." promptTitle="TIPO" prompt="Elige de la lista: CLASE, SESION, TRABAJO, ENTREGA o FORO." type="list">
-      <formula1>"CLASE,SESION,TRABAJO,ENTREGA,FORO"</formula1>
+    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige CLASE, SESION, TRABAJO, CUESTIONARIO o FORO." promptTitle="TIPO" prompt="Elige de la lista: CLASE, SESION, TRABAJO, CUESTIONARIO o FORO." type="list">
+      <formula1>"CLASE,SESION,TRABAJO,CUESTIONARIO,FORO"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Escribe la fecha como dd/mm/aaaa, por ejemplo 05/10/2026." promptTitle="FECHA" prompt="Formato dd/mm/aaaa. Ejemplo: 05/10/2026." type="date" operator="between">
       <formula1>DATE(2020,1,1)</formula1>
@@ -7812,7 +7812,7 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>CLASE o SESION = sesión (azul). TRABAJO o ENTREGA = entrega (naranja). FORO = foro (violeta), con hora límite como una entrega.</t>
+          <t>CLASE o SESION = sesión (azul). TRABAJO = trabajo (naranja). CUESTIONARIO = cuestionario o examen (verde). FORO = foro (violeta). Los tres usan hora límite.</t>
         </is>
       </c>
     </row>
@@ -8101,12 +8101,12 @@
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>ENTREGA</t>
+          <t>CUESTIONARIO</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Informe de lectura</t>
+          <t>Quiz unidad 2</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -8210,7 +8210,7 @@
       <c r="E34" s="16" t="n"/>
       <c r="F34" s="17" t="inlineStr">
         <is>
-          <t>Usa solo CLASE, SESION, TRABAJO, ENTREGA o FORO.</t>
+          <t>Usa solo CLASE, SESION, TRABAJO, CUESTIONARIO o FORO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Divide Clases y sesiones en Sesiones y Grabaciones
- Nuevo tipo GRABACION (rosa, ícono de pantalla con play): material disponible
  desde una fecha, hora opcional, botón «Ver grabación», no vence y no aparece
  en Próximas actividades. Filtro, leyenda y detalle propios.
- CLASE pasa a ser SESION: se acepta en Excel/editor con aviso y se guarda como SESION.
- Base de datos: categoría GRABACION, restricciones y función de importación
  actualizadas; eventos CLASE existentes se convierten (con hash recalculado).
- Plantilla, README y pruebas actualizadas (27 pruebas).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQGbJzWknhnvewuJZUfHUT
</commit_message>
<xml_diff>
--- a/public/plantilla-calendario.xlsx
+++ b/public/plantilla-calendario.xlsx
@@ -7634,8 +7634,8 @@
   </sheetData>
   <autoFilter ref="A1:H1001"/>
   <dataValidations count="7">
-    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige CLASE, SESION, TRABAJO, CUESTIONARIO o FORO." promptTitle="TIPO" prompt="Elige de la lista: CLASE, SESION, TRABAJO, CUESTIONARIO o FORO." type="list">
-      <formula1>"CLASE,SESION,TRABAJO,CUESTIONARIO,FORO"</formula1>
+    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige SESION, GRABACION, TRABAJO, CUESTIONARIO o FORO." promptTitle="TIPO" prompt="Elige de la lista: SESION, GRABACION, TRABAJO, CUESTIONARIO o FORO." type="list">
+      <formula1>"SESION,GRABACION,TRABAJO,CUESTIONARIO,FORO"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Escribe la fecha como dd/mm/aaaa, por ejemplo 05/10/2026." promptTitle="FECHA" prompt="Formato dd/mm/aaaa. Ejemplo: 05/10/2026." type="date" operator="between">
       <formula1>DATE(2020,1,1)</formula1>
@@ -7807,12 +7807,12 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>CLASE</t>
+          <t>SESION</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>CLASE o SESION = sesión (azul). TRABAJO = trabajo (naranja). CUESTIONARIO = cuestionario o examen (verde). FORO = foro (violeta). Los tres usan hora límite.</t>
+          <t>SESION = sesión en vivo (azul). GRABACION = grabación disponible desde su fecha (rosa). TRABAJO (naranja), CUESTIONARIO (verde) y FORO (violeta) usan hora límite.</t>
         </is>
       </c>
     </row>
@@ -8020,7 +8020,7 @@
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>CLASE</t>
+          <t>SESION</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -8047,22 +8047,22 @@
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>SESION</t>
+          <t>GRABACION</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Tutoría de proyecto</t>
+          <t>Grabación: Matemáticas II</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026 · 10:00 – 12:00</t>
+          <t>05/10/2026 · sin hora</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>https://zoom.us/j/123 · Revisión de avances</t>
+          <t>https://youtu.be/abc · Clase del 5 de octubre</t>
         </is>
       </c>
     </row>
@@ -8210,7 +8210,7 @@
       <c r="E34" s="16" t="n"/>
       <c r="F34" s="17" t="inlineStr">
         <is>
-          <t>Usa solo CLASE, SESION, TRABAJO, CUESTIONARIO o FORO.</t>
+          <t>Usa solo SESION, GRABACION, TRABAJO, CUESTIONARIO o FORO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sesiones Zajuna, Sesiones adicionales y nuevo tipo Dudas
- SESION se divide en SESION_ZAJUNA (prioritaria: azul intenso, etiqueta
  «Prioritaria», va primero a igual hora) y SESION_ADICIONAL (cian), con la
  misma cámara como ícono.
- Nuevo tipo DUDAS (ámbar, globo de chat con «?»): en vivo con horario,
  botón «Ir al chat de dudas» cuando tenga enlace.
- Homologación: SESION y CLASE se aceptan con aviso y se guardan como
  SESION_ZAJUNA; los 6 eventos SESION existentes pasan a SESION_ZAJUNA.
- Excel/editor aceptan «Sesión Zajuna», «sesion adicional», etc.
- Base de datos, plantilla, README y pruebas actualizadas (30 pruebas).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQGbJzWknhnvewuJZUfHUT
</commit_message>
<xml_diff>
--- a/public/plantilla-calendario.xlsx
+++ b/public/plantilla-calendario.xlsx
@@ -64,7 +64,7 @@
       <color rgb="00211F18"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -78,12 +78,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E3ECFB"/>
+        <fgColor rgb="00DCE6FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDF3F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF0D2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBE1EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FBEBDC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDF3E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -172,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -206,9 +226,21 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -580,7 +612,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -7634,14 +7666,14 @@
   </sheetData>
   <autoFilter ref="A1:H1001"/>
   <dataValidations count="7">
-    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige SESION, GRABACION, TRABAJO, CUESTIONARIO o FORO." promptTitle="TIPO" prompt="Elige de la lista: SESION, GRABACION, TRABAJO, CUESTIONARIO o FORO." type="list">
-      <formula1>"SESION,GRABACION,TRABAJO,CUESTIONARIO,FORO"</formula1>
+    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, TRABAJO, CUESTIONARIO o FORO." promptTitle="TIPO" prompt="Elige de la lista: SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, TRABAJO, CUESTIONARIO o FORO." type="list">
+      <formula1>"SESION_ZAJUNA,SESION_ADICIONAL,DUDAS,GRABACION,TRABAJO,CUESTIONARIO,FORO"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Escribe la fecha como dd/mm/aaaa, por ejemplo 05/10/2026." promptTitle="FECHA" prompt="Formato dd/mm/aaaa. Ejemplo: 05/10/2026." type="date" operator="between">
       <formula1>DATE(2020,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
     </dataValidation>
-    <dataValidation sqref="E2:F1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Hora no válida" error="Escribe la hora en formato 24 h, por ejemplo 08:00 o 14:30." promptTitle="HORA" prompt="Formato 24 h (08:00, 14:30). Obligatoria en clases. En trabajos es la hora límite." type="time" operator="between">
+    <dataValidation sqref="E2:F1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Hora no válida" error="Escribe la hora en formato 24 h, por ejemplo 08:00 o 14:30." promptTitle="HORA" prompt="Formato 24 h (08:00, 14:30). Obligatoria en sesiones y dudas. En trabajos es la hora límite." type="time" operator="between">
       <formula1>TIME(0,0,0)</formula1>
       <formula2>TIME(23,59,59)</formula2>
     </dataValidation>
@@ -7651,7 +7683,7 @@
     <dataValidation sqref="A2:A1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="ID_EVENTO" prompt="Déjalo vacío en filas nuevas: el sistema asigna el ID. No cambies los ID existentes." type="custom">
       <formula1>TRUE</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="LINK" prompt="Enlace de la sesión (https://...). Opcional." type="custom">
+    <dataValidation sqref="G2:G1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="LINK" prompt="Enlace de la sesión, del chat de dudas o del recurso (https://...). Opcional." type="custom">
       <formula1>TRUE</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="DESCRIPCION" prompt="Información adicional. Opcional. Máximo 2.000 caracteres." type="custom">
@@ -7668,7 +7700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F37"/>
+  <dimension ref="B2:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -7689,7 +7721,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Llena la hoja «Calendario» con TODAS las clases, sesiones, trabajos y entregas. Una fila por actividad. No cambies los nombres de las columnas ni el nombre de la hoja.</t>
+          <t>Llena la hoja «Calendario» con TODAS las sesiones, espacios de dudas, grabaciones, trabajos, cuestionarios y foros. Una fila por actividad. No cambies los nombres de las columnas ni el nombre de la hoja.</t>
         </is>
       </c>
     </row>
@@ -7807,12 +7839,12 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>SESION</t>
+          <t>SESION_ZAJUNA</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>SESION = sesión en vivo (azul). GRABACION = grabación disponible desde su fecha (rosa). TRABAJO (naranja), CUESTIONARIO (verde) y FORO (violeta) usan hora límite.</t>
+          <t>SESION_ZAJUNA = sesión Zajuna, prioritaria (azul intenso). SESION_ADICIONAL = sesión adicional (cian). DUDAS = espacio de dudas por chat (ámbar). Las tres son en vivo con hora de inicio. GRABACION = grabación disponible desde su fecha (rosa). TRABAJO (naranja), CUESTIONARIO (verde) y FORO (violeta) usan hora límite.</t>
         </is>
       </c>
     </row>
@@ -7866,7 +7898,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Fecha de la clase o de la entrega.</t>
+          <t>Fecha de la sesión, del espacio de dudas o de la entrega.</t>
         </is>
       </c>
     </row>
@@ -7878,7 +7910,7 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Sí en clases</t>
+          <t>Sí en sesiones y dudas</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -7920,7 +7952,7 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>Solo para clases. Debe ser posterior a la hora de inicio. Sin hora fin, la clase se considera de 1 hora.</t>
+          <t>Solo para sesiones y dudas. Debe ser posterior a la hora de inicio. Sin hora fin, se considera de 1 hora.</t>
         </is>
       </c>
     </row>
@@ -7947,7 +7979,7 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>Solo para clases. Sin enlace, la clase se publica sin botón «Ingresar».</t>
+          <t>Sesiones: botón «Ingresar a la sesión». Dudas: botón «Ir al chat de dudas» (agrégalo cuando se tenga). Sin enlace se publica sin botón.</t>
         </is>
       </c>
     </row>
@@ -8020,7 +8052,7 @@
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>SESION</t>
+          <t>SESION_ZAJUNA</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -8035,225 +8067,279 @@
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>https://meet.google.com/abc · Unidad 3</t>
+          <t>https://zajuna.sena.edu.co/… · Unidad 3</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>(vacío)</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>SESION_ADICIONAL</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Refuerzo de Matemáticas</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>06/10/2026 · 18:00 – 19:00</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>https://meet.google.com/abc</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>(vacío)</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>DUDAS</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Resolución de dudas</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>07/10/2026 · 19:00 – 20:00</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>Enlace al chat cuando se tenga</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>(vacío)</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>GRABACION</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Grabación: Matemáticas II</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>05/10/2026 · sin hora</t>
         </is>
       </c>
-      <c r="F25" s="12" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
         <is>
           <t>https://youtu.be/abc · Clase del 5 de octubre</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="13" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>EVT-0002</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>TRABAJO</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>Taller 2</t>
         </is>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>06/10/2026 · 23:59</t>
         </is>
       </c>
-      <c r="F26" s="13" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>Subir en PDF</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="13" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>(vacío)</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
         <is>
           <t>CUESTIONARIO</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>Quiz unidad 2</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
         <is>
           <t>08/10/2026 · sin hora</t>
         </is>
       </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="F29" s="17" t="inlineStr">
         <is>
           <t>Vence a las 11:59 PM de ese día</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="14" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>(vacío)</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>FORO</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
         <is>
           <t>Foro: la complejidad de la vida</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
         <is>
           <t>07/03/2027 · 23:59</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="F30" s="18" t="inlineStr">
         <is>
           <t>Participación en el foro de la plataforma</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="8" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Errores frecuentes</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="10" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Problema</t>
         </is>
       </c>
-      <c r="C31" s="15" t="n"/>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="n"/>
+      <c r="E33" s="20" t="n"/>
+      <c r="F33" s="10" t="inlineStr">
         <is>
           <t>Cómo corregirlo</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="17" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="21" t="inlineStr">
         <is>
           <t>Fecha como 35/15/2026</t>
         </is>
       </c>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="16" t="n"/>
-      <c r="F32" s="17" t="inlineStr">
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="20" t="n"/>
+      <c r="F34" s="21" t="inlineStr">
         <is>
           <t>Revisa día y mes. Debe ser una fecha real en formato dd/mm/aaaa.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="17" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="21" t="inlineStr">
         <is>
           <t>ID_EVENTO repetido</t>
         </is>
       </c>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="17" t="inlineStr">
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="20" t="n"/>
+      <c r="F35" s="21" t="inlineStr">
         <is>
           <t>Cada ID aparece una sola vez. En filas nuevas deja la celda vacía.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="17" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="21" t="inlineStr">
         <is>
           <t>Tipo «REUNION»</t>
         </is>
       </c>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="17" t="inlineStr">
-        <is>
-          <t>Usa solo SESION, GRABACION, TRABAJO, CUESTIONARIO o FORO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>Clase sin hora de inicio</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="n"/>
-      <c r="D35" s="15" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="17" t="inlineStr">
-        <is>
-          <t>Las clases y sesiones necesitan HORA_INICIO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="17" t="inlineStr">
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+      <c r="E36" s="20" t="n"/>
+      <c r="F36" s="21" t="inlineStr">
+        <is>
+          <t>Usa solo SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, TRABAJO, CUESTIONARIO o FORO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="21" t="inlineStr">
+        <is>
+          <t>Sesión o dudas sin hora de inicio</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="19" t="n"/>
+      <c r="E37" s="20" t="n"/>
+      <c r="F37" s="21" t="inlineStr">
+        <is>
+          <t>Las sesiones y los espacios de dudas necesitan HORA_INICIO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="21" t="inlineStr">
         <is>
           <t>Hora fin antes del inicio</t>
         </is>
       </c>
-      <c r="C36" s="15" t="n"/>
-      <c r="D36" s="15" t="n"/>
-      <c r="E36" s="16" t="n"/>
-      <c r="F36" s="17" t="inlineStr">
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="19" t="n"/>
+      <c r="E38" s="20" t="n"/>
+      <c r="F38" s="21" t="inlineStr">
         <is>
           <t>Corrige HORA_FIN o déjala vacía.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="B37" s="17" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="21" t="inlineStr">
         <is>
           <t>Link sin https://</t>
         </is>
       </c>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="17" t="inlineStr">
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="20" t="n"/>
+      <c r="F39" s="21" t="inlineStr">
         <is>
           <t>Copia el enlace completo, empezando por https://</t>
         </is>
@@ -8261,18 +8347,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B31:E31"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B35:E35"/>
     <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B34:E34"/>
     <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B38:E38"/>
     <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B39:E39"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B34:E34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Trabajos en rojo llamativo
- TRABAJO pasa de naranja a rojo (#ff4d57 oscuro / #e0182d claro).
- «Vence pronto» y los avisos conservan el naranja (nuevo token --warn)
  para no confundirse con el color de los trabajos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQGbJzWknhnvewuJZUfHUT
</commit_message>
<xml_diff>
--- a/public/plantilla-calendario.xlsx
+++ b/public/plantilla-calendario.xlsx
@@ -98,7 +98,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBEBDC"/>
+        <fgColor rgb="00FDDCDF"/>
       </patternFill>
     </fill>
     <fill>
@@ -7844,7 +7844,7 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>SESION_ZAJUNA = sesión Zajuna, prioritaria (azul intenso). SESION_ADICIONAL = sesión adicional (cian). DUDAS = espacio de dudas por chat (ámbar). Las tres son en vivo con hora de inicio. GRABACION = grabación disponible desde su fecha (rosa). TRABAJO (naranja), CUESTIONARIO (verde) y FORO (violeta) usan hora límite.</t>
+          <t>SESION_ZAJUNA = sesión Zajuna, prioritaria (azul intenso). SESION_ADICIONAL = sesión adicional (cian). DUDAS = espacio de dudas por chat (ámbar). Las tres son en vivo con hora de inicio. GRABACION = grabación disponible desde su fecha (rosa). TRABAJO (rojo), CUESTIONARIO (verde) y FORO (violeta) usan hora límite.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
«Trabajo» pasa a llamarse «Entrega» en toda la app y la base de datos
- Tipo TRABAJO → ENTREGA (filtro «Entregas», leyenda «Entrega», mensajes,
  plantilla, README). TRABAJO se sigue aceptando con aviso.
- ENTREGA deja de ser alias de CUESTIONARIO (ese cambio ya se aplicó).
- Base de datos: 27 eventos TRABAJO → ENTREGA; respaldos convertidos en
  orden (ENTREGA antiguo → CUESTIONARIO, luego TRABAJO → ENTREGA) para que
  «Deshacer» restaure cada tipo correctamente. Migración re-ejecutable.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQGbJzWknhnvewuJZUfHUT
</commit_message>
<xml_diff>
--- a/public/plantilla-calendario.xlsx
+++ b/public/plantilla-calendario.xlsx
@@ -7666,14 +7666,14 @@
   </sheetData>
   <autoFilter ref="A1:H1001"/>
   <dataValidations count="7">
-    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, TRABAJO, CUESTIONARIO o FORO." promptTitle="TIPO" prompt="Elige de la lista: SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, TRABAJO, CUESTIONARIO o FORO." type="list">
-      <formula1>"SESION_ZAJUNA,SESION_ADICIONAL,DUDAS,GRABACION,TRABAJO,CUESTIONARIO,FORO"</formula1>
+    <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, ENTREGA, CUESTIONARIO o FORO." promptTitle="TIPO" prompt="Elige de la lista: SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, ENTREGA, CUESTIONARIO o FORO." type="list">
+      <formula1>"SESION_ZAJUNA,SESION_ADICIONAL,DUDAS,GRABACION,ENTREGA,CUESTIONARIO,FORO"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Fecha no válida" error="Escribe la fecha como dd/mm/aaaa, por ejemplo 05/10/2026." promptTitle="FECHA" prompt="Formato dd/mm/aaaa. Ejemplo: 05/10/2026." type="date" operator="between">
       <formula1>DATE(2020,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
     </dataValidation>
-    <dataValidation sqref="E2:F1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Hora no válida" error="Escribe la hora en formato 24 h, por ejemplo 08:00 o 14:30." promptTitle="HORA" prompt="Formato 24 h (08:00, 14:30). Obligatoria en sesiones y dudas. En trabajos es la hora límite." type="time" operator="between">
+    <dataValidation sqref="E2:F1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Hora no válida" error="Escribe la hora en formato 24 h, por ejemplo 08:00 o 14:30." promptTitle="HORA" prompt="Formato 24 h (08:00, 14:30). Obligatoria en sesiones y dudas. En entregas es la hora límite." type="time" operator="between">
       <formula1>TIME(0,0,0)</formula1>
       <formula2>TIME(23,59,59)</formula2>
     </dataValidation>
@@ -7721,7 +7721,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Llena la hoja «Calendario» con TODAS las sesiones, espacios de dudas, grabaciones, trabajos, cuestionarios y foros. Una fila por actividad. No cambies los nombres de las columnas ni el nombre de la hoja.</t>
+          <t>Llena la hoja «Calendario» con TODAS las sesiones, espacios de dudas, grabaciones, entregas, cuestionarios y foros. Una fila por actividad. No cambies los nombres de las columnas ni el nombre de la hoja.</t>
         </is>
       </c>
     </row>
@@ -7844,7 +7844,7 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>SESION_ZAJUNA = sesión Zajuna, prioritaria (azul intenso). SESION_ADICIONAL = sesión adicional (cian). DUDAS = espacio de dudas por chat (ámbar). Las tres son en vivo con hora de inicio. GRABACION = grabación disponible desde su fecha (rosa). TRABAJO (rojo), CUESTIONARIO (verde) y FORO (violeta) usan hora límite.</t>
+          <t>SESION_ZAJUNA = sesión Zajuna, prioritaria (azul intenso). SESION_ADICIONAL = sesión adicional (cian). DUDAS = espacio de dudas por chat (ámbar). Las tres son en vivo con hora de inicio. GRABACION = grabación disponible desde su fecha (rosa). ENTREGA (rojo), CUESTIONARIO (verde) y FORO (violeta) usan hora límite.</t>
         </is>
       </c>
     </row>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>En trabajos es la hora límite. Si un trabajo no tiene hora, vence a las 11:59 PM.</t>
+          <t>En entregas es la hora límite. Si una entrega no tiene hora, vence a las 11:59 PM.</t>
         </is>
       </c>
     </row>
@@ -8160,7 +8160,7 @@
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>TRABAJO</t>
+          <t>ENTREGA</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr">
@@ -8296,7 +8296,7 @@
       <c r="E36" s="20" t="n"/>
       <c r="F36" s="21" t="inlineStr">
         <is>
-          <t>Usa solo SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, TRABAJO, CUESTIONARIO o FORO.</t>
+          <t>Usa solo SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, ENTREGA, CUESTIONARIO o FORO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Instructor en Sesiones Zajuna y Sesiones adicionales
- Nueva columna opcional INSTRUCTOR (Excel, plantilla y editor web).
  Solo aplica a SESION_ZAJUNA y SESION_ADICIONAL; en otros tipos se ignora
  con aviso. Excel sin la columna conserva los instructores guardados.
- Base de datos: events.instructor; la huella de contenido solo cambia si
  hay instructor (sin falsos «modificados»); importar, vista previa,
  historial y «Deshacer» lo incluyen.
- Calendario: instructor en Próximas actividades, detalle (o «Por
  confirmar») y Agenda. WhatsApp: en el resumen y en el aviso previo.
- Pegado sin encabezados detecta si la primera columna es TIPO o ID.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQGbJzWknhnvewuJZUfHUT
</commit_message>
<xml_diff>
--- a/public/plantilla-calendario.xlsx
+++ b/public/plantilla-calendario.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Calendario'!$A$1:$H$1001</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Calendario'!$A$1:$I$1001</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1001"/>
+  <dimension ref="A1:I1001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -619,6 +619,7 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -660,6 +661,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>DESCRIPCION</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>INSTRUCTOR</t>
         </is>
       </c>
     </row>
@@ -7664,8 +7670,8 @@
       <c r="H1001" s="5" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1001"/>
-  <dataValidations count="7">
+  <autoFilter ref="A1:I1001"/>
+  <dataValidations count="8">
     <dataValidation sqref="B2:B1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo no válido" error="Elige SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, ENTREGA, CUESTIONARIO o FORO." promptTitle="TIPO" prompt="Elige de la lista: SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, ENTREGA, CUESTIONARIO o FORO." type="list">
       <formula1>"SESION_ZAJUNA,SESION_ADICIONAL,DUDAS,GRABACION,ENTREGA,CUESTIONARIO,FORO"</formula1>
     </dataValidation>
@@ -7689,6 +7695,9 @@
     <dataValidation sqref="H2:H1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="DESCRIPCION" prompt="Información adicional. Opcional. Máximo 2.000 caracteres." type="custom">
       <formula1>TRUE</formula1>
     </dataValidation>
+    <dataValidation sqref="I2:I1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nombre muy largo" error="Máximo 120 caracteres." promptTitle="INSTRUCTOR" prompt="Persona que dicta la sesión. Opcional. Solo para SESION_ZAJUNA y SESION_ADICIONAL." type="textLength" operator="lessThanOrEqual">
+      <formula1>120</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7700,7 +7709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F39"/>
+  <dimension ref="B2:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8010,270 +8019,282 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="8" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>INSTRUCTOR</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Ana Pérez</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Quién dicta la sesión. Solo en SESION_ZAJUNA y SESION_ADICIONAL; en otros tipos se ignora. Máximo 120 caracteres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Ejemplos</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="10" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>ID_EVENTO</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>TIPO</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>NOMBRE</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>FECHA · HORAS</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F24" s="10" t="inlineStr">
         <is>
           <t>LINK / DESCRIPCIÓN</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="12" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>EVT-0001</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>SESION_ZAJUNA</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Matemáticas II</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>05/10/2026 · 08:00 – 10:00</t>
         </is>
       </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>https://zajuna.sena.edu.co/… · Unidad 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="13" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>https://zajuna.sena.edu.co/… · Unidad 3 · Instructor: Ana Pérez</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>(vacío)</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C26" s="13" t="inlineStr">
         <is>
           <t>SESION_ADICIONAL</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="D26" s="13" t="inlineStr">
         <is>
           <t>Refuerzo de Matemáticas</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="E26" s="13" t="inlineStr">
         <is>
           <t>06/10/2026 · 18:00 – 19:00</t>
         </is>
       </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="F26" s="13" t="inlineStr">
         <is>
           <t>https://meet.google.com/abc</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="14" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>(vacío)</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>DUDAS</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Resolución de dudas</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>07/10/2026 · 19:00 – 20:00</t>
         </is>
       </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>Enlace al chat cuando se tenga</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="15" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>(vacío)</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>GRABACION</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>Grabación: Matemáticas II</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>05/10/2026 · sin hora</t>
         </is>
       </c>
-      <c r="F27" s="15" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>https://youtu.be/abc · Clase del 5 de octubre</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="16" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>EVT-0002</t>
         </is>
       </c>
-      <c r="C28" s="16" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
         <is>
           <t>ENTREGA</t>
         </is>
       </c>
-      <c r="D28" s="16" t="inlineStr">
+      <c r="D29" s="16" t="inlineStr">
         <is>
           <t>Taller 2</t>
         </is>
       </c>
-      <c r="E28" s="16" t="inlineStr">
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>06/10/2026 · 23:59</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="F29" s="16" t="inlineStr">
         <is>
           <t>Subir en PDF</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="17" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>(vacío)</t>
         </is>
       </c>
-      <c r="C29" s="17" t="inlineStr">
+      <c r="C30" s="17" t="inlineStr">
         <is>
           <t>CUESTIONARIO</t>
         </is>
       </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>Quiz unidad 2</t>
         </is>
       </c>
-      <c r="E29" s="17" t="inlineStr">
+      <c r="E30" s="17" t="inlineStr">
         <is>
           <t>08/10/2026 · sin hora</t>
         </is>
       </c>
-      <c r="F29" s="17" t="inlineStr">
+      <c r="F30" s="17" t="inlineStr">
         <is>
           <t>Vence a las 11:59 PM de ese día</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="18" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="18" t="inlineStr">
         <is>
           <t>(vacío)</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>FORO</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="D31" s="18" t="inlineStr">
         <is>
           <t>Foro: la complejidad de la vida</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="E31" s="18" t="inlineStr">
         <is>
           <t>07/03/2027 · 23:59</t>
         </is>
       </c>
-      <c r="F30" s="18" t="inlineStr">
+      <c r="F31" s="18" t="inlineStr">
         <is>
           <t>Participación en el foro de la plataforma</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="8" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Errores frecuentes</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="10" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Problema</t>
-        </is>
-      </c>
-      <c r="C33" s="19" t="n"/>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="20" t="n"/>
-      <c r="F33" s="10" t="inlineStr">
-        <is>
-          <t>Cómo corregirlo</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="21" t="inlineStr">
-        <is>
-          <t>Fecha como 35/15/2026</t>
         </is>
       </c>
       <c r="C34" s="19" t="n"/>
       <c r="D34" s="19" t="n"/>
       <c r="E34" s="20" t="n"/>
-      <c r="F34" s="21" t="inlineStr">
-        <is>
-          <t>Revisa día y mes. Debe ser una fecha real en formato dd/mm/aaaa.</t>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>Cómo corregirlo</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="21" t="inlineStr">
         <is>
-          <t>ID_EVENTO repetido</t>
+          <t>Fecha como 35/15/2026</t>
         </is>
       </c>
       <c r="C35" s="19" t="n"/>
@@ -8281,14 +8302,14 @@
       <c r="E35" s="20" t="n"/>
       <c r="F35" s="21" t="inlineStr">
         <is>
-          <t>Cada ID aparece una sola vez. En filas nuevas deja la celda vacía.</t>
+          <t>Revisa día y mes. Debe ser una fecha real en formato dd/mm/aaaa.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="21" t="inlineStr">
         <is>
-          <t>Tipo «REUNION»</t>
+          <t>ID_EVENTO repetido</t>
         </is>
       </c>
       <c r="C36" s="19" t="n"/>
@@ -8296,14 +8317,14 @@
       <c r="E36" s="20" t="n"/>
       <c r="F36" s="21" t="inlineStr">
         <is>
-          <t>Usa solo SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, ENTREGA, CUESTIONARIO o FORO.</t>
+          <t>Cada ID aparece una sola vez. En filas nuevas deja la celda vacía.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="21" t="inlineStr">
         <is>
-          <t>Sesión o dudas sin hora de inicio</t>
+          <t>Tipo «REUNION»</t>
         </is>
       </c>
       <c r="C37" s="19" t="n"/>
@@ -8311,14 +8332,14 @@
       <c r="E37" s="20" t="n"/>
       <c r="F37" s="21" t="inlineStr">
         <is>
-          <t>Las sesiones y los espacios de dudas necesitan HORA_INICIO.</t>
+          <t>Usa solo SESION_ZAJUNA, SESION_ADICIONAL, DUDAS, GRABACION, ENTREGA, CUESTIONARIO o FORO.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="21" t="inlineStr">
         <is>
-          <t>Hora fin antes del inicio</t>
+          <t>Sesión o dudas sin hora de inicio</t>
         </is>
       </c>
       <c r="C38" s="19" t="n"/>
@@ -8326,14 +8347,14 @@
       <c r="E38" s="20" t="n"/>
       <c r="F38" s="21" t="inlineStr">
         <is>
-          <t>Corrige HORA_FIN o déjala vacía.</t>
+          <t>Las sesiones y los espacios de dudas necesitan HORA_INICIO.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="21" t="inlineStr">
         <is>
-          <t>Link sin https://</t>
+          <t>Hora fin antes del inicio</t>
         </is>
       </c>
       <c r="C39" s="19" t="n"/>
@@ -8341,19 +8362,34 @@
       <c r="E39" s="20" t="n"/>
       <c r="F39" s="21" t="inlineStr">
         <is>
+          <t>Corrige HORA_FIN o déjala vacía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>Link sin https://</t>
+        </is>
+      </c>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+      <c r="E40" s="20" t="n"/>
+      <c r="F40" s="21" t="inlineStr">
+        <is>
           <t>Copia el enlace completo, empezando por https://</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B40:E40"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B35:E35"/>
     <mergeCell ref="B37:E37"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B33:E33"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B9:F9"/>

</xml_diff>

<commit_message>
Instructor también en Grabaciones; duplicados distinguen instructor
- GRABACION acepta INSTRUCTOR (la grabación lleva el de la sesión grabada;
  el mismo instructor puede repetirse el mismo día). Se ve en el detalle.
- Dos sesiones con el mismo nombre, fecha y hora pero instructores
  distintos ya no se marcan como duplicadas.
- Base de datos, plantilla, README y pruebas (35) actualizadas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQGbJzWknhnvewuJZUfHUT
</commit_message>
<xml_diff>
--- a/public/plantilla-calendario.xlsx
+++ b/public/plantilla-calendario.xlsx
@@ -7695,7 +7695,7 @@
     <dataValidation sqref="H2:H1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="DESCRIPCION" prompt="Información adicional. Opcional. Máximo 2.000 caracteres." type="custom">
       <formula1>TRUE</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nombre muy largo" error="Máximo 120 caracteres." promptTitle="INSTRUCTOR" prompt="Persona que dicta la sesión. Opcional. Solo para SESION_ZAJUNA y SESION_ADICIONAL." type="textLength" operator="lessThanOrEqual">
+    <dataValidation sqref="I2:I1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nombre muy largo" error="Máximo 120 caracteres." promptTitle="INSTRUCTOR" prompt="Persona que dicta la sesión. Opcional. Para SESION_ZAJUNA, SESION_ADICIONAL y GRABACION." type="textLength" operator="lessThanOrEqual">
       <formula1>120</formula1>
     </dataValidation>
   </dataValidations>
@@ -8042,7 +8042,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>Quién dicta la sesión. Solo en SESION_ZAJUNA y SESION_ADICIONAL; en otros tipos se ignora. Máximo 120 caracteres.</t>
+          <t>Quién dicta la sesión. En SESION_ZAJUNA, SESION_ADICIONAL y GRABACION (la grabación lleva el instructor de la sesión; puede repetirse el mismo día); en otros tipos se ignora. Máximo 120 caracteres.</t>
         </is>
       </c>
     </row>
@@ -8184,7 +8184,7 @@
       </c>
       <c r="F28" s="15" t="inlineStr">
         <is>
-          <t>https://youtu.be/abc · Clase del 5 de octubre</t>
+          <t>https://youtu.be/abc · Clase del 5 de octubre · Instructor: Ana Pérez</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Instructor en cualquier sesión (también Dudas)
El instructor se acepta en SESION_ZAJUNA, SESION_ADICIONAL, DUDAS y
GRABACION, aunque coincidan fecha y hora. Solo entregas, cuestionarios
y foros lo ignoran con aviso. Base de datos actualizada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MQGbJzWknhnvewuJZUfHUT
</commit_message>
<xml_diff>
--- a/public/plantilla-calendario.xlsx
+++ b/public/plantilla-calendario.xlsx
@@ -7695,7 +7695,7 @@
     <dataValidation sqref="H2:H1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="DESCRIPCION" prompt="Información adicional. Opcional. Máximo 2.000 caracteres." type="custom">
       <formula1>TRUE</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nombre muy largo" error="Máximo 120 caracteres." promptTitle="INSTRUCTOR" prompt="Persona que dicta la sesión. Opcional. Para SESION_ZAJUNA, SESION_ADICIONAL y GRABACION." type="textLength" operator="lessThanOrEqual">
+    <dataValidation sqref="I2:I1001" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Nombre muy largo" error="Máximo 120 caracteres." promptTitle="INSTRUCTOR" prompt="Persona que dicta la sesión. Opcional. Para SESION_ZAJUNA, SESION_ADICIONAL, DUDAS y GRABACION." type="textLength" operator="lessThanOrEqual">
       <formula1>120</formula1>
     </dataValidation>
   </dataValidations>
@@ -8042,7 +8042,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>Quién dicta la sesión. En SESION_ZAJUNA, SESION_ADICIONAL y GRABACION (la grabación lleva el instructor de la sesión; puede repetirse el mismo día); en otros tipos se ignora. Máximo 120 caracteres.</t>
+          <t>Quién dicta la sesión. En cualquier sesión (SESION_ZAJUNA, SESION_ADICIONAL, DUDAS) y GRABACION (la grabación lleva el instructor de la sesión; puede repetirse el mismo día); en otros tipos se ignora. Máximo 120 caracteres.</t>
         </is>
       </c>
     </row>

</xml_diff>